<commit_message>
update ga4 changes deploy
</commit_message>
<xml_diff>
--- a/Pinterest-Distribution-Plan.xlsx
+++ b/Pinterest-Distribution-Plan.xlsx
@@ -16,6 +16,7 @@
     <sheet name="Pin Formats + AI Prompts" sheetId="6" state="visible" r:id="rId8"/>
     <sheet name="Scorecard" sheetId="7" state="visible" r:id="rId9"/>
     <sheet name="Tools &amp; Budget" sheetId="8" state="visible" r:id="rId10"/>
+    <sheet name="Pin Batch 1" sheetId="9" state="visible" r:id="rId11"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="404">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="578" uniqueCount="472">
   <si>
     <t xml:space="preserve">Pinterest Distribution Strategy - travelsamericas.com</t>
   </si>
@@ -1239,6 +1240,210 @@
   </si>
   <si>
     <t xml:space="preserve">At 50-60 pins/month = $1-2 per pin all-in</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pin Batch 1 — Week 3 (12 pins, schedule 2/day)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Workflow per pin: open template SVG -&gt; replace placeholders with Title (split across the two title lines) -&gt; export PNG 1000x1500 -&gt; upload to Pinterest -&gt; paste Title, Description, URL exactly -&gt; assign Board -&gt; schedule. Mark Status when queued.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pin ID (utm_content)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Template</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Board</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pin Title</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pin Description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Destination URL (paste exactly)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">checklist-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 Checklist</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NYC Safety Tips</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NYC Safety Checklist: 7 Habits for First-Time Visitors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Practical NYC safety tips for tourists — subway habits, scam awareness, and smart night-walking rules from a street-tested New York City safety guide. Save this checklist for your trip.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.travelsamericas.com/destination/nyc/nyc-safety-guide?utm_source=pinterest&amp;utm_medium=organic&amp;utm_campaign=safety&amp;utm_content=checklist-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">checklist-02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NYC Subway + Getting Around</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NYC Subway at Night: 5 Rules I Always Follow</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Riding the NYC subway alone at night? These 5 subway safety rules — where to stand, which car to pick, late-night transfer tips — keep solo travelers confident.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.travelsamericas.com/destination/nyc/subway-safety-guide?utm_source=pinterest&amp;utm_medium=organic&amp;utm_campaign=safety&amp;utm_content=checklist-02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">checklist-03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NYC Solo Female Travel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Solo Female Travel NYC: Pre-Trip Safety Setup</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Traveling to New York alone? 5 things to set up before you land — location sharing, backup payments, and the safety apps worth having. From our NYC solo female travel guide.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.travelsamericas.com/destination/nyc/nyc-female-solo-travel-guide?utm_source=pinterest&amp;utm_medium=organic&amp;utm_campaign=safety&amp;utm_content=checklist-03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">checklist-04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Is NYC Safe at Night? 5 Things to Know</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Walking NYC at night as a tourist: which areas stay busy, when to switch to rideshare, and the after-dark rules locals actually use. Honest night-safety breakdown.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.travelsamericas.com/destination/nyc/is-nyc-safe-at-night?utm_source=pinterest&amp;utm_medium=organic&amp;utm_campaign=safety&amp;utm_content=checklist-04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">itinerary-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4 Itinerary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NYC Itineraries</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 Days in NYC Alone: An Itinerary That Works</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A realistic 3-day NYC itinerary for solo travelers — Central Park to the Brooklyn Bridge, with solo-friendly food stops and budget notes. Free printable PDF included.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.travelsamericas.com/destination/nyc/solo-itinerary?utm_source=pinterest&amp;utm_medium=organic&amp;utm_campaign=planning&amp;utm_content=itinerary-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">itinerary-02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Solo Trip to NYC: The First-Timer’s Plan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Planning a solo trip to New York City? Where to stay, how to ride the subway with confidence, daily budgets, and a 3-day plan — built for first-time solo travelers.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.travelsamericas.com/destination/nyc/solo-trip-to-nyc?utm_source=pinterest&amp;utm_medium=organic&amp;utm_campaign=solo&amp;utm_content=itinerary-02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">itinerary-03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Your First 24 Hours in NYC, Solo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The arrival-day plan that prevents day-one burnout: transit from JFK, a 30-minute orientation loop, and the easiest first solo dinner in New York City.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.travelsamericas.com/destination/nyc/solo-trip-to-nyc?utm_source=pinterest&amp;utm_medium=organic&amp;utm_campaign=solo&amp;utm_content=itinerary-03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">listicle-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 Listicle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Where to Stay in NYC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7 Safest Areas to Stay in NYC, Compared</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Where to stay in NYC as a solo traveler: 7 neighborhoods compared for safety, late-night walkability, and subway access — with the hotel zones worth paying for.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.travelsamericas.com/destination/nyc/best-areas-to-stay?utm_source=pinterest&amp;utm_medium=organic&amp;utm_campaign=insider&amp;utm_content=listicle-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">map-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 Map</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NYC After Dark: Walk Here, Ride There</t>
+  </si>
+  <si>
+    <t xml:space="preserve">An honest NYC neighborhood safety map for visitors — where streets stay lively at night, where to stay alert, and where a rideshare beats walking. Block-by-block guide.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.travelsamericas.com/destination/nyc/neighborhood-guide?utm_source=pinterest&amp;utm_medium=organic&amp;utm_campaign=insider&amp;utm_content=map-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">listicle-02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Where to Stay in NYC: First Solo Trip Edition</t>
+  </si>
+  <si>
+    <t xml:space="preserve">First solo trip to New York? Stay between 14th and 96th in Manhattan, within 5 minutes of a subway line — plus 3 rules for picking a safe hotel block.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.travelsamericas.com/destination/nyc/best-areas-to-stay?utm_source=pinterest&amp;utm_medium=organic&amp;utm_campaign=insider&amp;utm_content=listicle-02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pdf-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Free PDF: 3-Day NYC Solo Itinerary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grab the free printable NYC itinerary — day-by-day plan, packing list, and budget breakdown, sent instantly. Made for first-time solo travelers to New York City.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.travelsamericas.com/destination/nyc/solo-itinerary?utm_source=pinterest&amp;utm_medium=organic&amp;utm_campaign=planning&amp;utm_content=pdf-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pdf-02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5 Stat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Solo Travel Tips for Women</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NYC Packing List + 3-Day Plan (Free PDF)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What to pack for New York plus a complete 3-day solo plan in one free PDF — walking-shoe rules, subway payment tips, and a realistic budget table. Sent instantly.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.travelsamericas.com/destination/nyc/solo-itinerary?utm_source=pinterest&amp;utm_medium=organic&amp;utm_campaign=planning&amp;utm_content=pdf-02</t>
   </si>
 </sst>
 </file>
@@ -1411,7 +1616,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="30">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1520,20 +1725,16 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -3963,14 +4164,14 @@
       <c r="G23" s="25"/>
       <c r="H23" s="25"/>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="27" t="s">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="24" t="s">
         <v>350</v>
       </c>
-      <c r="B25" s="28"/>
+      <c r="B25" s="27"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="29" t="s">
+      <c r="A26" s="26" t="s">
         <v>351</v>
       </c>
       <c r="B26" s="25" t="s">
@@ -3987,7 +4188,7 @@
       <c r="K26" s="25"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="29" t="s">
+      <c r="A27" s="26" t="s">
         <v>353</v>
       </c>
       <c r="B27" s="25" t="s">
@@ -4004,7 +4205,7 @@
       <c r="K27" s="25"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="29" t="s">
+      <c r="A28" s="26" t="s">
         <v>355</v>
       </c>
       <c r="B28" s="25" t="s">
@@ -4021,7 +4222,7 @@
       <c r="K28" s="25"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="29" t="s">
+      <c r="A29" s="26" t="s">
         <v>357</v>
       </c>
       <c r="B29" s="25" t="s">
@@ -4038,7 +4239,7 @@
       <c r="K29" s="25"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="29" t="s">
+      <c r="A30" s="26" t="s">
         <v>359</v>
       </c>
       <c r="B30" s="25" t="s">
@@ -4055,7 +4256,7 @@
       <c r="K30" s="25"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="29" t="s">
+      <c r="A31" s="26" t="s">
         <v>361</v>
       </c>
       <c r="B31" s="25" t="s">
@@ -4071,8 +4272,8 @@
       <c r="J31" s="25"/>
       <c r="K31" s="25"/>
     </row>
-    <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="29" t="s">
+    <row r="32" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="26" t="s">
         <v>363</v>
       </c>
       <c r="B32" s="25" t="s">
@@ -4089,7 +4290,7 @@
       <c r="K32" s="25"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="29" t="s">
+      <c r="A33" s="26" t="s">
         <v>365</v>
       </c>
       <c r="B33" s="25" t="s">
@@ -4292,10 +4493,10 @@
       <c r="A10" s="4" t="s">
         <v>400</v>
       </c>
-      <c r="B10" s="30" t="s">
+      <c r="B10" s="28" t="s">
         <v>401</v>
       </c>
-      <c r="C10" s="30" t="s">
+      <c r="C10" s="28" t="s">
         <v>402</v>
       </c>
       <c r="D10" s="4" t="s">
@@ -4314,4 +4515,367 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:H15"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="70"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="29" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="10" t="s">
+        <v>405</v>
+      </c>
+      <c r="B2" s="10"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
+      <c r="G2" s="10"/>
+      <c r="H2" s="10"/>
+    </row>
+    <row r="3" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>406</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>407</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>408</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>409</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>410</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>411</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>418</v>
+      </c>
+      <c r="H4" s="6"/>
+    </row>
+    <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>419</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>414</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>420</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>421</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>422</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>423</v>
+      </c>
+      <c r="H5" s="5"/>
+    </row>
+    <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>424</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>425</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>426</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>427</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>428</v>
+      </c>
+      <c r="H6" s="6"/>
+    </row>
+    <row r="7" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>429</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>414</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>415</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>430</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>431</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>432</v>
+      </c>
+      <c r="H7" s="5"/>
+    </row>
+    <row r="8" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>433</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>434</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>435</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>436</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>437</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>438</v>
+      </c>
+      <c r="H8" s="6"/>
+    </row>
+    <row r="9" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>434</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>425</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>440</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>441</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>442</v>
+      </c>
+      <c r="H9" s="5"/>
+    </row>
+    <row r="10" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>443</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>434</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>435</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>444</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>445</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>446</v>
+      </c>
+      <c r="H10" s="6"/>
+    </row>
+    <row r="11" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>447</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>448</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>449</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>450</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>451</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>452</v>
+      </c>
+      <c r="H11" s="5"/>
+    </row>
+    <row r="12" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>453</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>454</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>455</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>456</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>457</v>
+      </c>
+      <c r="H12" s="6"/>
+    </row>
+    <row r="13" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>458</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>448</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>449</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>459</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>460</v>
+      </c>
+      <c r="G13" s="5" t="s">
+        <v>461</v>
+      </c>
+      <c r="H13" s="5"/>
+    </row>
+    <row r="14" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>462</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>434</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>435</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>463</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>464</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>465</v>
+      </c>
+      <c r="H14" s="6"/>
+    </row>
+    <row r="15" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>466</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>467</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>468</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>469</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>470</v>
+      </c>
+      <c r="G15" s="5" t="s">
+        <v>471</v>
+      </c>
+      <c r="H15" s="5"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:H2"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>